<commit_message>
chore(planning): add named agent roster and Agents tab
Each agent is a persistent worker with a fixed model/effort; workbook
rows log against the agent's name.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/Hashirai Clearance POC - Plan.xlsx
+++ b/planning/Hashirai Clearance POC - Plan.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="Stories" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Tasks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Calibration" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Agents" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Calibration" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Summary" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stories'!$A$1:$O$13</definedName>
@@ -1737,7 +1738,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>implementer-T1.1</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -1822,7 +1823,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>implementer-T2.1</t>
+          <t>Mika</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
@@ -1907,7 +1908,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>implementer-T9.1</t>
+          <t>Quinn</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
@@ -1992,7 +1993,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>implementer-T1.2</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -2077,7 +2078,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>implementer-T3.1</t>
+          <t>Sasha</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
@@ -2162,7 +2163,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>implementer-T5.1</t>
+          <t>Ellis</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -2247,7 +2248,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>implementer-T8.1</t>
+          <t>Mika</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
@@ -2332,7 +2333,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>implementer-T10.1</t>
+          <t>Quinn</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
@@ -2417,7 +2418,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>implementer-T11.1</t>
+          <t>Remy</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
@@ -2502,7 +2503,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>implementer-T3.2</t>
+          <t>Sasha</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -2587,7 +2588,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>implementer-T4.1</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
@@ -2672,7 +2673,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>implementer-T5.2</t>
+          <t>Ellis</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
@@ -2757,7 +2758,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>implementer-T7.1</t>
+          <t>Jules</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
@@ -2842,7 +2843,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>implementer-T8.2</t>
+          <t>Mika</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -2927,7 +2928,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>implementer-T10.2</t>
+          <t>Quinn</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
@@ -3012,7 +3013,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>implementer-T11.2</t>
+          <t>Remy</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
@@ -3097,7 +3098,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>implementer-T3.3</t>
+          <t>Sasha</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -3186,7 +3187,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>implementer-T6.1</t>
+          <t>Noor</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
@@ -3275,7 +3276,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>implementer-T7.2</t>
+          <t>Remy</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
@@ -3360,7 +3361,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>implementer-T12.1</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
@@ -3445,7 +3446,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>implementer-T12.2</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
@@ -5085,6 +5086,658 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Multiplier</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Lane</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Tasks assigned</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Tasks accepted</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Rejected attempts</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Baseline SP</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Adjusted SP</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Runtime (min)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Raw actual SP</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Normalised actual SP</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Actual ÷ estimate (raw ÷ adjusted, accepted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Quinn</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D2" s="4">
+        <f>INDEX(Calibration!$D$5:$D$11,MATCH(B2&amp;" "&amp;C2,Calibration!$A$5:$A$11,0))</f>
+        <v/>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Policy and sidecar</t>
+        </is>
+      </c>
+      <c r="F2" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A2,Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="G2" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A2,Tasks!$S$2:$S$62,"Y")</f>
+        <v/>
+      </c>
+      <c r="H2" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A2,Tasks!$S$2:$S$62,"N")-COUNTIFS(Tasks!$D$2:$D$62,$A2,Tasks!$S$2:$S$62,"N",Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="I2" s="5">
+        <f>SUMIFS(Tasks!$I$2:$I$62,Tasks!$D$2:$D$62,$A2)</f>
+        <v/>
+      </c>
+      <c r="J2" s="5">
+        <f>SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A2)</f>
+        <v/>
+      </c>
+      <c r="K2" s="7">
+        <f>SUMIFS(Tasks!$P$2:$P$62,Tasks!$D$2:$D$62,$A2)</f>
+        <v/>
+      </c>
+      <c r="L2" s="5">
+        <f>SUMIFS(Tasks!$T$2:$T$62,Tasks!$D$2:$D$62,$A2)</f>
+        <v/>
+      </c>
+      <c r="M2" s="5">
+        <f>SUMIFS(Tasks!$U$2:$U$62,Tasks!$D$2:$D$62,$A2)</f>
+        <v/>
+      </c>
+      <c r="N2" s="4">
+        <f>IF(SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A2,Tasks!$S$2:$S$62,"Y")=0,"",L2/SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A2,Tasks!$S$2:$S$62,"Y"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Rowan</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D3" s="4">
+        <f>INDEX(Calibration!$D$5:$D$11,MATCH(B3&amp;" "&amp;C3,Calibration!$A$5:$A$11,0))</f>
+        <v/>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Platform: scaffold, CI, reset, agent, e2e</t>
+        </is>
+      </c>
+      <c r="F3" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A3,Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="G3" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A3,Tasks!$S$2:$S$62,"Y")</f>
+        <v/>
+      </c>
+      <c r="H3" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A3,Tasks!$S$2:$S$62,"N")-COUNTIFS(Tasks!$D$2:$D$62,$A3,Tasks!$S$2:$S$62,"N",Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="I3" s="5">
+        <f>SUMIFS(Tasks!$I$2:$I$62,Tasks!$D$2:$D$62,$A3)</f>
+        <v/>
+      </c>
+      <c r="J3" s="5">
+        <f>SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A3)</f>
+        <v/>
+      </c>
+      <c r="K3" s="7">
+        <f>SUMIFS(Tasks!$P$2:$P$62,Tasks!$D$2:$D$62,$A3)</f>
+        <v/>
+      </c>
+      <c r="L3" s="5">
+        <f>SUMIFS(Tasks!$T$2:$T$62,Tasks!$D$2:$D$62,$A3)</f>
+        <v/>
+      </c>
+      <c r="M3" s="5">
+        <f>SUMIFS(Tasks!$U$2:$U$62,Tasks!$D$2:$D$62,$A3)</f>
+        <v/>
+      </c>
+      <c r="N3" s="4">
+        <f>IF(SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A3,Tasks!$S$2:$S$62,"Y")=0,"",L3/SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A3,Tasks!$S$2:$S$62,"Y"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Sasha</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D4" s="4">
+        <f>INDEX(Calibration!$D$5:$D$11,MATCH(B4&amp;" "&amp;C4,Calibration!$A$5:$A$11,0))</f>
+        <v/>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="F4" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A4,Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="G4" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A4,Tasks!$S$2:$S$62,"Y")</f>
+        <v/>
+      </c>
+      <c r="H4" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A4,Tasks!$S$2:$S$62,"N")-COUNTIFS(Tasks!$D$2:$D$62,$A4,Tasks!$S$2:$S$62,"N",Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="I4" s="5">
+        <f>SUMIFS(Tasks!$I$2:$I$62,Tasks!$D$2:$D$62,$A4)</f>
+        <v/>
+      </c>
+      <c r="J4" s="5">
+        <f>SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A4)</f>
+        <v/>
+      </c>
+      <c r="K4" s="7">
+        <f>SUMIFS(Tasks!$P$2:$P$62,Tasks!$D$2:$D$62,$A4)</f>
+        <v/>
+      </c>
+      <c r="L4" s="5">
+        <f>SUMIFS(Tasks!$T$2:$T$62,Tasks!$D$2:$D$62,$A4)</f>
+        <v/>
+      </c>
+      <c r="M4" s="5">
+        <f>SUMIFS(Tasks!$U$2:$U$62,Tasks!$D$2:$D$62,$A4)</f>
+        <v/>
+      </c>
+      <c r="N4" s="4">
+        <f>IF(SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A4,Tasks!$S$2:$S$62,"Y")=0,"",L4/SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A4,Tasks!$S$2:$S$62,"Y"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Ellis</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D5" s="4">
+        <f>INDEX(Calibration!$D$5:$D$11,MATCH(B5&amp;" "&amp;C5,Calibration!$A$5:$A$11,0))</f>
+        <v/>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Classifier</t>
+        </is>
+      </c>
+      <c r="F5" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A5,Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="G5" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A5,Tasks!$S$2:$S$62,"Y")</f>
+        <v/>
+      </c>
+      <c r="H5" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A5,Tasks!$S$2:$S$62,"N")-COUNTIFS(Tasks!$D$2:$D$62,$A5,Tasks!$S$2:$S$62,"N",Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="I5" s="5">
+        <f>SUMIFS(Tasks!$I$2:$I$62,Tasks!$D$2:$D$62,$A5)</f>
+        <v/>
+      </c>
+      <c r="J5" s="5">
+        <f>SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A5)</f>
+        <v/>
+      </c>
+      <c r="K5" s="7">
+        <f>SUMIFS(Tasks!$P$2:$P$62,Tasks!$D$2:$D$62,$A5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="5">
+        <f>SUMIFS(Tasks!$T$2:$T$62,Tasks!$D$2:$D$62,$A5)</f>
+        <v/>
+      </c>
+      <c r="M5" s="5">
+        <f>SUMIFS(Tasks!$U$2:$U$62,Tasks!$D$2:$D$62,$A5)</f>
+        <v/>
+      </c>
+      <c r="N5" s="4">
+        <f>IF(SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A5,Tasks!$S$2:$S$62,"Y")=0,"",L5/SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A5,Tasks!$S$2:$S$62,"Y"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Jules</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D6" s="4">
+        <f>INDEX(Calibration!$D$5:$D$11,MATCH(B6&amp;" "&amp;C6,Calibration!$A$5:$A$11,0))</f>
+        <v/>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Poller</t>
+        </is>
+      </c>
+      <c r="F6" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A6,Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="G6" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A6,Tasks!$S$2:$S$62,"Y")</f>
+        <v/>
+      </c>
+      <c r="H6" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A6,Tasks!$S$2:$S$62,"N")-COUNTIFS(Tasks!$D$2:$D$62,$A6,Tasks!$S$2:$S$62,"N",Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="I6" s="5">
+        <f>SUMIFS(Tasks!$I$2:$I$62,Tasks!$D$2:$D$62,$A6)</f>
+        <v/>
+      </c>
+      <c r="J6" s="5">
+        <f>SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="7">
+        <f>SUMIFS(Tasks!$P$2:$P$62,Tasks!$D$2:$D$62,$A6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="5">
+        <f>SUMIFS(Tasks!$T$2:$T$62,Tasks!$D$2:$D$62,$A6)</f>
+        <v/>
+      </c>
+      <c r="M6" s="5">
+        <f>SUMIFS(Tasks!$U$2:$U$62,Tasks!$D$2:$D$62,$A6)</f>
+        <v/>
+      </c>
+      <c r="N6" s="4">
+        <f>IF(SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A6,Tasks!$S$2:$S$62,"Y")=0,"",L6/SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A6,Tasks!$S$2:$S$62,"Y"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Mika</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Sonnet 5.5</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D7" s="4">
+        <f>INDEX(Calibration!$D$5:$D$11,MATCH(B7&amp;" "&amp;C7,Calibration!$A$5:$A$11,0))</f>
+        <v/>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Seed data and decision log</t>
+        </is>
+      </c>
+      <c r="F7" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A7,Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="G7" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A7,Tasks!$S$2:$S$62,"Y")</f>
+        <v/>
+      </c>
+      <c r="H7" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A7,Tasks!$S$2:$S$62,"N")-COUNTIFS(Tasks!$D$2:$D$62,$A7,Tasks!$S$2:$S$62,"N",Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="I7" s="5">
+        <f>SUMIFS(Tasks!$I$2:$I$62,Tasks!$D$2:$D$62,$A7)</f>
+        <v/>
+      </c>
+      <c r="J7" s="5">
+        <f>SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="7">
+        <f>SUMIFS(Tasks!$P$2:$P$62,Tasks!$D$2:$D$62,$A7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="5">
+        <f>SUMIFS(Tasks!$T$2:$T$62,Tasks!$D$2:$D$62,$A7)</f>
+        <v/>
+      </c>
+      <c r="M7" s="5">
+        <f>SUMIFS(Tasks!$U$2:$U$62,Tasks!$D$2:$D$62,$A7)</f>
+        <v/>
+      </c>
+      <c r="N7" s="4">
+        <f>IF(SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A7,Tasks!$S$2:$S$62,"Y")=0,"",L7/SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A7,Tasks!$S$2:$S$62,"Y"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Remy</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Sonnet 5.5</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D8" s="4">
+        <f>INDEX(Calibration!$D$5:$D$11,MATCH(B8&amp;" "&amp;C8,Calibration!$A$5:$A$11,0))</f>
+        <v/>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Tools and npm start</t>
+        </is>
+      </c>
+      <c r="F8" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A8,Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="G8" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A8,Tasks!$S$2:$S$62,"Y")</f>
+        <v/>
+      </c>
+      <c r="H8" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A8,Tasks!$S$2:$S$62,"N")-COUNTIFS(Tasks!$D$2:$D$62,$A8,Tasks!$S$2:$S$62,"N",Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="I8" s="5">
+        <f>SUMIFS(Tasks!$I$2:$I$62,Tasks!$D$2:$D$62,$A8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="5">
+        <f>SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="7">
+        <f>SUMIFS(Tasks!$P$2:$P$62,Tasks!$D$2:$D$62,$A8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="5">
+        <f>SUMIFS(Tasks!$T$2:$T$62,Tasks!$D$2:$D$62,$A8)</f>
+        <v/>
+      </c>
+      <c r="M8" s="5">
+        <f>SUMIFS(Tasks!$U$2:$U$62,Tasks!$D$2:$D$62,$A8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="4">
+        <f>IF(SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A8,Tasks!$S$2:$S$62,"Y")=0,"",L8/SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A8,Tasks!$S$2:$S$62,"Y"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Noor</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D9" s="4">
+        <f>INDEX(Calibration!$D$5:$D$11,MATCH(B9&amp;" "&amp;C9,Calibration!$A$5:$A$11,0))</f>
+        <v/>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Fixture recording</t>
+        </is>
+      </c>
+      <c r="F9" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A9,Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="G9" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A9,Tasks!$S$2:$S$62,"Y")</f>
+        <v/>
+      </c>
+      <c r="H9" s="15">
+        <f>COUNTIFS(Tasks!$D$2:$D$62,$A9,Tasks!$S$2:$S$62,"N")-COUNTIFS(Tasks!$D$2:$D$62,$A9,Tasks!$S$2:$S$62,"N",Tasks!$I$2:$I$62,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="I9" s="5">
+        <f>SUMIFS(Tasks!$I$2:$I$62,Tasks!$D$2:$D$62,$A9)</f>
+        <v/>
+      </c>
+      <c r="J9" s="5">
+        <f>SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="7">
+        <f>SUMIFS(Tasks!$P$2:$P$62,Tasks!$D$2:$D$62,$A9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="5">
+        <f>SUMIFS(Tasks!$T$2:$T$62,Tasks!$D$2:$D$62,$A9)</f>
+        <v/>
+      </c>
+      <c r="M9" s="5">
+        <f>SUMIFS(Tasks!$U$2:$U$62,Tasks!$D$2:$D$62,$A9)</f>
+        <v/>
+      </c>
+      <c r="N9" s="4">
+        <f>IF(SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A9,Tasks!$S$2:$S$62,"Y")=0,"",L9/SUMIFS(Tasks!$M$2:$M$62,Tasks!$D$2:$D$62,$A9,Tasks!$S$2:$S$62,"Y"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8">
+        <f>SUM(F2:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="8">
+        <f>SUM(G2:G9)</f>
+        <v/>
+      </c>
+      <c r="H10" s="8">
+        <f>SUM(H2:H9)</f>
+        <v/>
+      </c>
+      <c r="I10" s="9">
+        <f>SUM(I2:I9)</f>
+        <v/>
+      </c>
+      <c r="J10" s="9">
+        <f>SUM(J2:J9)</f>
+        <v/>
+      </c>
+      <c r="K10" s="11">
+        <f>SUM(K2:K9)</f>
+        <v/>
+      </c>
+      <c r="L10" s="9">
+        <f>SUM(L2:L9)</f>
+        <v/>
+      </c>
+      <c r="M10" s="9">
+        <f>SUM(M2:M9)</f>
+        <v/>
+      </c>
+      <c r="N10" s="10" t="n"/>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Each agent is one persistent worker with a fixed model and effort; it keeps its lane across waves and is continued, not restarted, for its next task. Every Tasks row (including rejected attempts) names its agent in Owner agent.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A12:N12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5522,7 +6175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5551,7 +6204,7 @@
     <row r="2" ht="45" customHeight="1">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>How to use: fill in only the yellow cells on Tasks (Start, End, Attempts, PR link, Accepted, Notes) and on Stories (Status, Accepted). Log a rejected attempt on its own Tasks row: same ID, Story ID, Wave, Model and Effort, blank Baseline SP, Accepted = N, and the reason in Notes. Blue = typed-in value, black = formula, green = link to another tab.</t>
+          <t>How to use: fill in only the yellow cells on Tasks (Start, End, Attempts, PR link, Accepted, Notes) and on Stories (Status, Accepted). Log a rejected attempt on its own Tasks row: same ID, Story ID, Wave, Owner agent, Model and Effort, blank Baseline SP, Accepted = N, and the reason in Notes. Blue = typed-in value, black = formula, green = link to another tab.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(planning): record wave 1 actuals per agent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/Hashirai Clearance POC - Plan.xlsx
+++ b/planning/Hashirai Clearance POC - Plan.xlsx
@@ -121,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -192,6 +192,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -728,7 +731,7 @@
       </c>
       <c r="J2" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K2" s="6" t="inlineStr">
@@ -797,12 +800,12 @@
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L3" s="7">
@@ -1280,12 +1283,12 @@
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L10" s="7">
@@ -1551,6 +1554,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="12" t="inlineStr">
         <is>
@@ -1780,19 +1784,27 @@
         <f>IF(OR(I2="",L2=""),"",I2*L2)</f>
         <v/>
       </c>
-      <c r="N2" s="13" t="n"/>
-      <c r="O2" s="13" t="n"/>
+      <c r="N2" s="26" t="n">
+        <v>46314.51927083333</v>
+      </c>
+      <c r="O2" s="26" t="n">
+        <v>46314.52329861111</v>
+      </c>
       <c r="P2" s="7">
         <f>IF(AND(ISNUMBER(N2),ISNUMBER(O2)),ROUND((O2-N2)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q2" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/4</t>
+        </is>
+      </c>
       <c r="S2" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T2" s="5">
@@ -1803,7 +1815,11 @@
         <f>IF(OR(T2="",L2=""),"",T2/L2)</f>
         <v/>
       </c>
-      <c r="V2" s="14" t="inlineStr"/>
+      <c r="V2" s="6" t="inlineStr">
+        <is>
+          <t>Accepted. Combined wave-1 check: vitest 30/30, typecheck ok, policy 8/8.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1865,19 +1881,27 @@
         <f>IF(OR(I3="",L3=""),"",I3*L3)</f>
         <v/>
       </c>
-      <c r="N3" s="13" t="n"/>
-      <c r="O3" s="13" t="n"/>
+      <c r="N3" s="26" t="n">
+        <v>46314.52429398148</v>
+      </c>
+      <c r="O3" s="26" t="n">
+        <v>46314.52466435185</v>
+      </c>
       <c r="P3" s="7">
         <f>IF(AND(ISNUMBER(N3),ISNUMBER(O3)),ROUND((O3-N3)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="14" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="R3" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/2</t>
+        </is>
+      </c>
       <c r="S3" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T3" s="5">
@@ -1888,7 +1912,11 @@
         <f>IF(OR(T3="",L3=""),"",T3/L3)</f>
         <v/>
       </c>
-      <c r="V3" s="14" t="inlineStr"/>
+      <c r="V3" s="6" t="inlineStr">
+        <is>
+          <t>Accepted after rework (attempt 2). Runtime includes the rejected attempt row.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1950,19 +1978,27 @@
         <f>IF(OR(I4="",L4=""),"",I4*L4)</f>
         <v/>
       </c>
-      <c r="N4" s="13" t="n"/>
-      <c r="O4" s="13" t="n"/>
+      <c r="N4" s="26" t="n">
+        <v>46314.51925925926</v>
+      </c>
+      <c r="O4" s="26" t="n">
+        <v>46314.52314814815</v>
+      </c>
       <c r="P4" s="7">
         <f>IF(AND(ISNUMBER(N4),ISNUMBER(O4)),ROUND((O4-N4)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/3</t>
+        </is>
+      </c>
       <c r="S4" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T4" s="5">
@@ -1973,7 +2009,11 @@
         <f>IF(OR(T4="",L4=""),"",T4/L4)</f>
         <v/>
       </c>
-      <c r="V4" s="14" t="inlineStr"/>
+      <c r="V4" s="6" t="inlineStr">
+        <is>
+          <t>Accepted. Spike: array recipients via @rcpt:addr/$to work (no fallback). describe --check exit 0, replay 8/8 (orchestrator rerun).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3514,17 +3554,39 @@
       <c r="V22" s="14" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="n"/>
-      <c r="B23" s="15" t="n"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>T2.1</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
       <c r="C23" s="15" t="n"/>
-      <c r="D23" s="15" t="n"/>
-      <c r="E23" s="15" t="n"/>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Mika</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="F23" s="15" t="n"/>
       <c r="G23" s="15" t="n"/>
       <c r="H23" s="15" t="n"/>
       <c r="I23" s="5" t="n"/>
-      <c r="J23" s="15" t="n"/>
-      <c r="K23" s="15" t="n"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Sonnet 5.5</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
       <c r="L23" s="4">
         <f>IF(J23="","",INDEX(Calibration!$D$5:$D$11,MATCH(J23&amp;" "&amp;K23,Calibration!$A$5:$A$11,0)))</f>
         <v/>
@@ -3533,15 +3595,23 @@
         <f>IF(OR(I23="",L23=""),"",I23*L23)</f>
         <v/>
       </c>
-      <c r="N23" s="13" t="n"/>
-      <c r="O23" s="13" t="n"/>
+      <c r="N23" s="26" t="n">
+        <v>46314.51927083333</v>
+      </c>
+      <c r="O23" s="26" t="n">
+        <v>46314.52086805556</v>
+      </c>
       <c r="P23" s="7">
         <f>IF(AND(ISNUMBER(N23),ISNUMBER(O23)),ROUND((O23-N23)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q23" s="14" t="n"/>
       <c r="R23" s="14" t="n"/>
-      <c r="S23" s="14" t="n"/>
+      <c r="S23" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="T23" s="5">
         <f>IF(S23="Y",SUMIFS($P$2:$P$62,$A$2:$A$62,A23&amp;"")/20,"")</f>
         <v/>
@@ -3550,7 +3620,11 @@
         <f>IF(OR(T23="",L23=""),"",T23/L23)</f>
         <v/>
       </c>
-      <c r="V23" s="14" t="n"/>
+      <c r="V23" s="6" t="inlineStr">
+        <is>
+          <t>Rejected attempt 1: tsc TS2345 at seed.test.ts:50 (only visible once T1.1's TypeScript was applied).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n"/>
@@ -6697,7 +6771,6 @@
       </c>
       <c r="H18" s="8" t="n"/>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="19" t="inlineStr">
         <is>
@@ -6944,7 +7017,6 @@
         <v/>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
         <is>
@@ -7077,13 +7149,6 @@
           <t>Per-value taint, so external sends of unrelated values after a Legal read are allowed.</t>
         </is>
       </c>
-      <c r="B35" s="25" t="n"/>
-      <c r="C35" s="25" t="n"/>
-      <c r="D35" s="25" t="n"/>
-      <c r="E35" s="25" t="n"/>
-      <c r="F35" s="25" t="n"/>
-      <c r="G35" s="25" t="n"/>
-      <c r="H35" s="25" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="25" t="inlineStr">
@@ -7091,13 +7156,6 @@
           <t>Per-record memory labels, instead of scoped audiences.</t>
         </is>
       </c>
-      <c r="B36" s="25" t="n"/>
-      <c r="C36" s="25" t="n"/>
-      <c r="D36" s="25" t="n"/>
-      <c r="E36" s="25" t="n"/>
-      <c r="F36" s="25" t="n"/>
-      <c r="G36" s="25" t="n"/>
-      <c r="H36" s="25" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="25" t="inlineStr">
@@ -7105,13 +7163,6 @@
           <t>An LLM-driven agent instead of the scripted one.</t>
         </is>
       </c>
-      <c r="B37" s="25" t="n"/>
-      <c r="C37" s="25" t="n"/>
-      <c r="D37" s="25" t="n"/>
-      <c r="E37" s="25" t="n"/>
-      <c r="F37" s="25" t="n"/>
-      <c r="G37" s="25" t="n"/>
-      <c r="H37" s="25" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="25" t="inlineStr">
@@ -7119,13 +7170,6 @@
           <t>A release workflow or UI for the review hold, beyond moving the file in Drive.</t>
         </is>
       </c>
-      <c r="B38" s="25" t="n"/>
-      <c r="C38" s="25" t="n"/>
-      <c r="D38" s="25" t="n"/>
-      <c r="E38" s="25" t="n"/>
-      <c r="F38" s="25" t="n"/>
-      <c r="G38" s="25" t="n"/>
-      <c r="H38" s="25" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="25" t="inlineStr">
@@ -7133,13 +7177,6 @@
           <t>Real ID detectors (SSN, passport and so on) beyond the SPECIMEN format.</t>
         </is>
       </c>
-      <c r="B39" s="25" t="n"/>
-      <c r="C39" s="25" t="n"/>
-      <c r="D39" s="25" t="n"/>
-      <c r="E39" s="25" t="n"/>
-      <c r="F39" s="25" t="n"/>
-      <c r="G39" s="25" t="n"/>
-      <c r="H39" s="25" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="25" t="inlineStr">
@@ -7147,13 +7184,6 @@
           <t>Google Docs, PDF and OCR input.</t>
         </is>
       </c>
-      <c r="B40" s="25" t="n"/>
-      <c r="C40" s="25" t="n"/>
-      <c r="D40" s="25" t="n"/>
-      <c r="E40" s="25" t="n"/>
-      <c r="F40" s="25" t="n"/>
-      <c r="G40" s="25" t="n"/>
-      <c r="H40" s="25" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="25" t="inlineStr">
@@ -7161,13 +7191,6 @@
           <t>Per-team audiences (an Accounting list separate from `internal`).</t>
         </is>
       </c>
-      <c r="B41" s="25" t="n"/>
-      <c r="C41" s="25" t="n"/>
-      <c r="D41" s="25" t="n"/>
-      <c r="E41" s="25" t="n"/>
-      <c r="F41" s="25" t="n"/>
-      <c r="G41" s="25" t="n"/>
-      <c r="H41" s="25" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="25" t="inlineStr">
@@ -7175,13 +7198,6 @@
           <t>Copies and summaries carrying the source clearance, and sanitizers or redaction.</t>
         </is>
       </c>
-      <c r="B42" s="25" t="n"/>
-      <c r="C42" s="25" t="n"/>
-      <c r="D42" s="25" t="n"/>
-      <c r="E42" s="25" t="n"/>
-      <c r="F42" s="25" t="n"/>
-      <c r="G42" s="25" t="n"/>
-      <c r="H42" s="25" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="25" t="inlineStr">
@@ -7189,13 +7205,6 @@
           <t>Real email.</t>
         </is>
       </c>
-      <c r="B43" s="25" t="n"/>
-      <c r="C43" s="25" t="n"/>
-      <c r="D43" s="25" t="n"/>
-      <c r="E43" s="25" t="n"/>
-      <c r="F43" s="25" t="n"/>
-      <c r="G43" s="25" t="n"/>
-      <c r="H43" s="25" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="25" t="inlineStr">
@@ -7203,13 +7212,6 @@
           <t>Drive webhooks.</t>
         </is>
       </c>
-      <c r="B44" s="25" t="n"/>
-      <c r="C44" s="25" t="n"/>
-      <c r="D44" s="25" t="n"/>
-      <c r="E44" s="25" t="n"/>
-      <c r="F44" s="25" t="n"/>
-      <c r="G44" s="25" t="n"/>
-      <c r="H44" s="25" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="25" t="inlineStr">
@@ -7217,13 +7219,6 @@
           <t>Reclassifying a file when it is edited.</t>
         </is>
       </c>
-      <c r="B45" s="25" t="n"/>
-      <c r="C45" s="25" t="n"/>
-      <c r="D45" s="25" t="n"/>
-      <c r="E45" s="25" t="n"/>
-      <c r="F45" s="25" t="n"/>
-      <c r="G45" s="25" t="n"/>
-      <c r="H45" s="25" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="25" t="inlineStr">
@@ -7231,13 +7226,6 @@
           <t>Hashirai Registry integration.</t>
         </is>
       </c>
-      <c r="B46" s="25" t="n"/>
-      <c r="C46" s="25" t="n"/>
-      <c r="D46" s="25" t="n"/>
-      <c r="E46" s="25" t="n"/>
-      <c r="F46" s="25" t="n"/>
-      <c r="G46" s="25" t="n"/>
-      <c r="H46" s="25" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="25" t="inlineStr">
@@ -7245,13 +7233,6 @@
           <t>A decision-log viewer.</t>
         </is>
       </c>
-      <c r="B47" s="25" t="n"/>
-      <c r="C47" s="25" t="n"/>
-      <c r="D47" s="25" t="n"/>
-      <c r="E47" s="25" t="n"/>
-      <c r="F47" s="25" t="n"/>
-      <c r="G47" s="25" t="n"/>
-      <c r="H47" s="25" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="25" t="inlineStr">
@@ -7259,19 +7240,11 @@
           <t>Retries, rate limits and deployment.</t>
         </is>
       </c>
-      <c r="B48" s="25" t="n"/>
-      <c r="C48" s="25" t="n"/>
-      <c r="D48" s="25" t="n"/>
-      <c r="E48" s="25" t="n"/>
-      <c r="F48" s="25" t="n"/>
-      <c r="G48" s="25" t="n"/>
-      <c r="H48" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A39:H39"/>
-    <mergeCell ref="A46:H46"/>
     <mergeCell ref="A35:H35"/>
     <mergeCell ref="A43:H43"/>
     <mergeCell ref="A38:H38"/>
@@ -7282,6 +7255,7 @@
     <mergeCell ref="A44:H44"/>
     <mergeCell ref="A47:H47"/>
     <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A46:H46"/>
     <mergeCell ref="A37:H37"/>
     <mergeCell ref="A40:H40"/>
   </mergeCells>

</xml_diff>

<commit_message>
chore(planning): record wave 2 actuals per agent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/Hashirai Clearance POC - Plan.xlsx
+++ b/planning/Hashirai Clearance POC - Plan.xlsx
@@ -869,7 +869,7 @@
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -2160,19 +2160,27 @@
         <f>IF(OR(I6="",L6=""),"",I6*L6)</f>
         <v/>
       </c>
-      <c r="N6" s="13" t="n"/>
-      <c r="O6" s="13" t="n"/>
+      <c r="N6" s="26" t="n">
+        <v>46314.54443287037</v>
+      </c>
+      <c r="O6" s="26" t="n">
+        <v>46314.54755787037</v>
+      </c>
       <c r="P6" s="7">
         <f>IF(AND(ISNUMBER(N6),ISNUMBER(O6)),ROUND((O6-N6)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/9</t>
+        </is>
+      </c>
       <c r="S6" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T6" s="5">
@@ -2183,7 +2191,11 @@
         <f>IF(OR(T6="",L6=""),"",T6/L6)</f>
         <v/>
       </c>
-      <c r="V6" s="14" t="inlineStr"/>
+      <c r="V6" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: in scope (5 files), contract suite runs on fake and Google stub, trash is soft (trashed=true), DriveScopeError outside the tree. Combined wave-2 check passed (128/128).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2245,19 +2257,27 @@
         <f>IF(OR(I7="",L7=""),"",I7*L7)</f>
         <v/>
       </c>
-      <c r="N7" s="13" t="n"/>
-      <c r="O7" s="13" t="n"/>
+      <c r="N7" s="26" t="n">
+        <v>46314.54443287037</v>
+      </c>
+      <c r="O7" s="26" t="n">
+        <v>46314.54645833333</v>
+      </c>
       <c r="P7" s="7">
         <f>IF(AND(ISNUMBER(N7),ISNUMBER(O7)),ROUND((O7-N7)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R7" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/8</t>
+        </is>
+      </c>
       <c r="S7" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T7" s="5">
@@ -2268,7 +2288,11 @@
         <f>IF(OR(T7="",L7=""),"",T7/L7)</f>
         <v/>
       </c>
-      <c r="V7" s="14" t="inlineStr"/>
+      <c r="V7" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: in scope (6 files), file name never reaches Jev (tested). Minor: commit 6798f8d0 doesn't typecheck alone (imports a file from the next commit); tip is fine.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2330,19 +2354,27 @@
         <f>IF(OR(I8="",L8=""),"",I8*L8)</f>
         <v/>
       </c>
-      <c r="N8" s="13" t="n"/>
-      <c r="O8" s="13" t="n"/>
+      <c r="N8" s="26" t="n">
+        <v>46314.54399305556</v>
+      </c>
+      <c r="O8" s="26" t="n">
+        <v>46314.54462962963</v>
+      </c>
       <c r="P8" s="7">
         <f>IF(AND(ISNUMBER(N8),ISNUMBER(O8)),ROUND((O8-N8)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/6</t>
+        </is>
+      </c>
       <c r="S8" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T8" s="5">
@@ -2353,7 +2385,11 @@
         <f>IF(OR(T8="",L8=""),"",T8/L8)</f>
         <v/>
       </c>
-      <c r="V8" s="14" t="inlineStr"/>
+      <c r="V8" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: in scope (2 files), exact-string tests of demo-script lines; combined wave-2 check passed (128/128).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2415,19 +2451,27 @@
         <f>IF(OR(I9="",L9=""),"",I9*L9)</f>
         <v/>
       </c>
-      <c r="N9" s="13" t="n"/>
-      <c r="O9" s="13" t="n"/>
+      <c r="N9" s="26" t="n">
+        <v>46314.5440162037</v>
+      </c>
+      <c r="O9" s="26" t="n">
+        <v>46314.54840277778</v>
+      </c>
       <c r="P9" s="7">
         <f>IF(AND(ISNUMBER(N9),ISNUMBER(O9)),ROUND((O9-N9)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/10</t>
+        </is>
+      </c>
       <c r="S9" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T9" s="5">
@@ -2438,7 +2482,11 @@
         <f>IF(OR(T9="",L9=""),"",T9/L9)</f>
         <v/>
       </c>
-      <c r="V9" s="14" t="inlineStr"/>
+      <c r="V9" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: live remedy flow against real appa; combined wave-2 check 128/128 incl. live, typecheck ok, policy 8/8. Live feedback wording differs from replay (T10.2 must use recorded fixtures).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2500,19 +2548,27 @@
         <f>IF(OR(I10="",L10=""),"",I10*L10)</f>
         <v/>
       </c>
-      <c r="N10" s="13" t="n"/>
-      <c r="O10" s="13" t="n"/>
+      <c r="N10" s="26" t="n">
+        <v>46314.54444444444</v>
+      </c>
+      <c r="O10" s="26" t="n">
+        <v>46314.54555555555</v>
+      </c>
       <c r="P10" s="7">
         <f>IF(AND(ISNUMBER(N10),ISNUMBER(O10)),ROUND((O10-N10)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R10" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/7</t>
+        </is>
+      </c>
       <c r="S10" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T10" s="5">
@@ -2523,7 +2579,11 @@
         <f>IF(OR(T10="",L10=""),"",T10/L10)</f>
         <v/>
       </c>
-      <c r="V10" s="14" t="inlineStr"/>
+      <c r="V10" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: in scope (4 files), no APPA calls, outbox written via schema orderKeys; combined wave-2 check passed (128/128). PR body end time 13:06:00Z is slightly off; real end used.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(planning): log T1.2 actuals; wave 2 merged
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/Hashirai Clearance POC - Plan.xlsx
+++ b/planning/Hashirai Clearance POC - Plan.xlsx
@@ -731,12 +731,12 @@
       </c>
       <c r="J2" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L2" s="7">
@@ -2075,19 +2075,27 @@
         <f>IF(OR(I5="",L5=""),"",I5*L5)</f>
         <v/>
       </c>
-      <c r="N5" s="13" t="n"/>
-      <c r="O5" s="13" t="n"/>
+      <c r="N5" s="26" t="n">
+        <v>46314.5519212963</v>
+      </c>
+      <c r="O5" s="26" t="n">
+        <v>46314.55635416666</v>
+      </c>
       <c r="P5" s="7">
         <f>IF(AND(ISNUMBER(N5),ISNUMBER(O5)),ROUND((O5-N5)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R5" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/11</t>
+        </is>
+      </c>
       <c r="S5" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T5" s="5">
@@ -2098,7 +2106,11 @@
         <f>IF(OR(T5="",L5=""),"",T5/L5)</f>
         <v/>
       </c>
-      <c r="V5" s="14" t="inlineStr"/>
+      <c r="V5" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: CI green cold (4m31s) and cached (19s, cache hit); check clearance-ci now required on main. Blocked 9.7 min waiting for Soham's workflow scope: wall-clock End-Start includes that; active time 8.1 min.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3687,17 +3699,39 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="n"/>
-      <c r="B24" s="15" t="n"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>T1.2</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Rowan</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="F24" s="15" t="n"/>
       <c r="G24" s="15" t="n"/>
       <c r="H24" s="15" t="n"/>
       <c r="I24" s="5" t="n"/>
-      <c r="J24" s="15" t="n"/>
-      <c r="K24" s="15" t="n"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
       <c r="L24" s="4">
         <f>IF(J24="","",INDEX(Calibration!$D$5:$D$11,MATCH(J24&amp;" "&amp;K24,Calibration!$A$5:$A$11,0)))</f>
         <v/>
@@ -3706,8 +3740,12 @@
         <f>IF(OR(I24="",L24=""),"",I24*L24)</f>
         <v/>
       </c>
-      <c r="N24" s="13" t="n"/>
-      <c r="O24" s="13" t="n"/>
+      <c r="N24" s="26" t="n">
+        <v>46314.54398148148</v>
+      </c>
+      <c r="O24" s="26" t="n">
+        <v>46314.54516203704</v>
+      </c>
       <c r="P24" s="7">
         <f>IF(AND(ISNUMBER(N24),ISNUMBER(O24)),ROUND((O24-N24)*1440,1),"")</f>
         <v/>
@@ -3723,7 +3761,11 @@
         <f>IF(OR(T24="",L24=""),"",T24/L24)</f>
         <v/>
       </c>
-      <c r="V24" s="14" t="n"/>
+      <c r="V24" s="6" t="inlineStr">
+        <is>
+          <t>Earlier work segment of the accepted attempt (paused while blocked).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="n"/>

</xml_diff>

<commit_message>
chore(planning): log waves 3-4 per agent; demo-script corrections
Fixture covers the 9 Jev files; guarded list line; seed 10 at 0.66;
OAuth decided. Later list gains poller durability, seed-10 margin and
reset speed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/Hashirai Clearance POC - Plan.xlsx
+++ b/planning/Hashirai Clearance POC - Plan.xlsx
@@ -869,12 +869,12 @@
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L4" s="7">
@@ -938,12 +938,12 @@
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L5" s="7">
@@ -1007,12 +1007,12 @@
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L6" s="7">
@@ -1076,12 +1076,12 @@
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L7" s="7">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -1352,12 +1352,12 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L11" s="7">
@@ -1421,12 +1421,12 @@
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L12" s="7">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
@@ -2270,21 +2270,21 @@
         <v/>
       </c>
       <c r="N7" s="26" t="n">
-        <v>46314.54443287037</v>
+        <v>46314.57232638889</v>
       </c>
       <c r="O7" s="26" t="n">
-        <v>46314.54645833333</v>
+        <v>46314.57354166666</v>
       </c>
       <c r="P7" s="7">
         <f>IF(AND(ISNUMBER(N7),ISNUMBER(O7)),ROUND((O7-N7)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R7" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/soham956/OpenAPPA/pull/8</t>
+          <t>https://github.com/soham956/OpenAPPA/pull/8 + #23 (rework)</t>
         </is>
       </c>
       <c r="S7" s="6" t="inlineStr">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="V7" s="6" t="inlineStr">
         <is>
-          <t>Accepted: in scope (6 files), file name never reaches Jev (tested). Minor: commit 6798f8d0 doesn't typecheck alone (imports a file from the next commit); tip is fine.</t>
+          <t>Accepted after rework (PR #23): fixture built from seed files at test time, no writes to committed files. Original PR #8 work counted as the rejected attempt row.</t>
         </is>
       </c>
     </row>
@@ -2657,19 +2657,27 @@
         <f>IF(OR(I11="",L11=""),"",I11*L11)</f>
         <v/>
       </c>
-      <c r="N11" s="13" t="n"/>
-      <c r="O11" s="13" t="n"/>
+      <c r="N11" s="26" t="n">
+        <v>46314.56222222222</v>
+      </c>
+      <c r="O11" s="26" t="n">
+        <v>46314.56504629629</v>
+      </c>
       <c r="P11" s="7">
         <f>IF(AND(ISNUMBER(N11),ISNUMBER(O11)),ROUND((O11-N11)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/19</t>
+        </is>
+      </c>
       <c r="S11" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T11" s="5">
@@ -2680,7 +2688,11 @@
         <f>IF(OR(T11="",L11=""),"",T11/L11)</f>
         <v/>
       </c>
-      <c r="V11" s="14" t="inlineStr"/>
+      <c r="V11" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: CI green, 16 tests with stubs, PKCE loopback consent (127.0.0.1), token mode 600, no live run. Combined wave-3 check 220/220.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2742,19 +2754,27 @@
         <f>IF(OR(I12="",L12=""),"",I12*L12)</f>
         <v/>
       </c>
-      <c r="N12" s="13" t="n"/>
-      <c r="O12" s="13" t="n"/>
+      <c r="N12" s="26" t="n">
+        <v>46314.56222222222</v>
+      </c>
+      <c r="O12" s="26" t="n">
+        <v>46314.56444444445</v>
+      </c>
       <c r="P12" s="7">
         <f>IF(AND(ISNUMBER(N12),ISNUMBER(O12)),ROUND((O12-N12)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R12" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/17</t>
+        </is>
+      </c>
       <c r="S12" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T12" s="5">
@@ -2765,7 +2785,11 @@
         <f>IF(OR(T12="",L12=""),"",T12/L12)</f>
         <v/>
       </c>
-      <c r="V12" s="14" t="inlineStr"/>
+      <c r="V12" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: in scope, CI green, 13 tests on fake incl. outsideTreeIds()=[] and sidecar refusal. Real Drive factory not yet wired (TODO(T3.2) seam) - wiring scheduled for wave 4. Combined wave-3 check 220/220.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2827,19 +2851,27 @@
         <f>IF(OR(I13="",L13=""),"",I13*L13)</f>
         <v/>
       </c>
-      <c r="N13" s="13" t="n"/>
-      <c r="O13" s="13" t="n"/>
+      <c r="N13" s="26" t="n">
+        <v>46314.56222222222</v>
+      </c>
+      <c r="O13" s="26" t="n">
+        <v>46314.56482638889</v>
+      </c>
       <c r="P13" s="7">
         <f>IF(AND(ISNUMBER(N13),ISNUMBER(O13)),ROUND((O13-N13)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R13" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/18</t>
+        </is>
+      </c>
       <c r="S13" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T13" s="5">
@@ -2850,7 +2882,11 @@
         <f>IF(OR(T13="",L13=""),"",T13/L13)</f>
         <v/>
       </c>
-      <c r="V13" s="14" t="inlineStr"/>
+      <c r="V13" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: CI green, each commit builds, SDK mocked, content-only. Orchestrator ruling: fixture holds 9 entries (08/09 never reach Jev - ID rule first); demo-script wording to be corrected.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2912,19 +2948,27 @@
         <f>IF(OR(I14="",L14=""),"",I14*L14)</f>
         <v/>
       </c>
-      <c r="N14" s="13" t="n"/>
-      <c r="O14" s="13" t="n"/>
+      <c r="N14" s="26" t="n">
+        <v>46314.56241898148</v>
+      </c>
+      <c r="O14" s="26" t="n">
+        <v>46314.56422453704</v>
+      </c>
       <c r="P14" s="7">
         <f>IF(AND(ISNUMBER(N14),ISNUMBER(O14)),ROUND((O14-N14)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R14" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/16</t>
+        </is>
+      </c>
       <c r="S14" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T14" s="5">
@@ -2935,7 +2979,11 @@
         <f>IF(OR(T14="",L14=""),"",T14/L14)</f>
         <v/>
       </c>
-      <c r="V14" s="14" t="inlineStr"/>
+      <c r="V14" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: in scope (2 files), CI green, 9 tests incl. restart/retry. Known edge: a log-write failure after a successful move loses that classify line (noted for T7.2). Combined wave-3 check 220/220.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2997,19 +3045,27 @@
         <f>IF(OR(I15="",L15=""),"",I15*L15)</f>
         <v/>
       </c>
-      <c r="N15" s="13" t="n"/>
-      <c r="O15" s="13" t="n"/>
+      <c r="N15" s="26" t="n">
+        <v>46314.56224537037</v>
+      </c>
+      <c r="O15" s="26" t="n">
+        <v>46314.56439814815</v>
+      </c>
       <c r="P15" s="7">
         <f>IF(AND(ISNUMBER(N15),ISNUMBER(O15)),ROUND((O15-N15)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R15" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/15</t>
+        </is>
+      </c>
       <c r="S15" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T15" s="5">
@@ -3020,7 +3076,11 @@
         <f>IF(OR(T15="",L15=""),"",T15/L15)</f>
         <v/>
       </c>
-      <c r="V15" s="14" t="inlineStr"/>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: in scope (4 files), CI green, 18 tests; reasons checked against demo-script text. Combined wave-3 check 220/220.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3082,19 +3142,27 @@
         <f>IF(OR(I16="",L16=""),"",I16*L16)</f>
         <v/>
       </c>
-      <c r="N16" s="13" t="n"/>
-      <c r="O16" s="13" t="n"/>
+      <c r="N16" s="26" t="n">
+        <v>46314.5622337963</v>
+      </c>
+      <c r="O16" s="26" t="n">
+        <v>46314.5671412037</v>
+      </c>
       <c r="P16" s="7">
         <f>IF(AND(ISNUMBER(N16),ISNUMBER(O16)),ROUND((O16-N16)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R16" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/20</t>
+        </is>
+      </c>
       <c r="S16" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T16" s="5">
@@ -3105,7 +3173,11 @@
         <f>IF(OR(T16="",L16=""),"",T16/L16)</f>
         <v/>
       </c>
-      <c r="V16" s="14" t="inlineStr"/>
+      <c r="V16" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: exact 2a/2b/2c reasons live + replayed from fixtures; denied tools never run; CI ran live guard tests. Combined wave-3 check 220/220. Has its own default drive tools - T12.1 to inject T11.2's.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -3167,19 +3239,27 @@
         <f>IF(OR(I17="",L17=""),"",I17*L17)</f>
         <v/>
       </c>
-      <c r="N17" s="13" t="n"/>
-      <c r="O17" s="13" t="n"/>
+      <c r="N17" s="26" t="n">
+        <v>46314.56225694445</v>
+      </c>
+      <c r="O17" s="26" t="n">
+        <v>46314.56357638889</v>
+      </c>
       <c r="P17" s="7">
         <f>IF(AND(ISNUMBER(N17),ISNUMBER(O17)),ROUND((O17-N17)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R17" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/14</t>
+        </is>
+      </c>
       <c r="S17" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T17" s="5">
@@ -3190,7 +3270,11 @@
         <f>IF(OR(T17="",L17=""),"",T17/L17)</f>
         <v/>
       </c>
-      <c r="V17" s="14" t="inlineStr"/>
+      <c r="V17" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: in scope (2 files), CI green, no APPA calls, DriveScopeError outside tree. Combined wave-3 check 220/220.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -3252,19 +3336,27 @@
         <f>IF(OR(I18="",L18=""),"",I18*L18)</f>
         <v/>
       </c>
-      <c r="N18" s="13" t="n"/>
-      <c r="O18" s="13" t="n"/>
+      <c r="N18" s="26" t="n">
+        <v>46314.57548611111</v>
+      </c>
+      <c r="O18" s="26" t="n">
+        <v>46314.57783564815</v>
+      </c>
       <c r="P18" s="7">
         <f>IF(AND(ISNUMBER(N18),ISNUMBER(O18)),ROUND((O18-N18)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R18" s="6" t="inlineStr">
+        <is>
+          <t>(no PR - verification only, no fixes needed)</t>
+        </is>
+      </c>
       <c r="S18" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T18" s="5">
@@ -3277,7 +3369,7 @@
       </c>
       <c r="V18" s="6" t="inlineStr">
         <is>
-          <t>Needs external inputs (see tasks.md). Moved from wave 5 to wave 4 by the orchestrator.</t>
+          <t>Accepted: live drive:check without browser, reset x3 + drop on real Workspace Drive, step 0 state verified, no fixes. Reset ~23-45s (don't run live mid-demo). Consent click done by Soham (not agent time). Orchestrator verified git status clean.</t>
         </is>
       </c>
     </row>
@@ -3341,19 +3433,27 @@
         <f>IF(OR(I19="",L19=""),"",I19*L19)</f>
         <v/>
       </c>
-      <c r="N19" s="13" t="n"/>
-      <c r="O19" s="13" t="n"/>
+      <c r="N19" s="26" t="n">
+        <v>46314.57394675926</v>
+      </c>
+      <c r="O19" s="26" t="n">
+        <v>46314.57481481481</v>
+      </c>
       <c r="P19" s="7">
         <f>IF(AND(ISNUMBER(N19),ISNUMBER(O19)),ROUND((O19-N19)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R19" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/25</t>
+        </is>
+      </c>
       <c r="S19" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T19" s="5">
@@ -3366,7 +3466,7 @@
       </c>
       <c r="V19" s="6" t="inlineStr">
         <is>
-          <t>Needs external inputs (see tasks.md). Moved from wave 5 to wave 4 by the orchestrator.</t>
+          <t>Accepted: 9-entry fixture (01-07,11 at 1.0; 10 Legal 0.66 -&gt; low-confidence), 3 live runs, seed 10 edited, no secrets, CI green. Paused while T5.1 test fix landed (not Noor's defect).</t>
         </is>
       </c>
     </row>
@@ -3430,19 +3530,27 @@
         <f>IF(OR(I20="",L20=""),"",I20*L20)</f>
         <v/>
       </c>
-      <c r="N20" s="13" t="n"/>
-      <c r="O20" s="13" t="n"/>
+      <c r="N20" s="26" t="n">
+        <v>46314.56958333333</v>
+      </c>
+      <c r="O20" s="26" t="n">
+        <v>46314.57119212963</v>
+      </c>
       <c r="P20" s="7">
         <f>IF(AND(ISNUMBER(N20),ISNUMBER(O20)),ROUND((O20-N20)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R20" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/22</t>
+        </is>
+      </c>
       <c r="S20" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T20" s="5">
@@ -3453,7 +3561,11 @@
         <f>IF(OR(T20="",L20=""),"",T20/L20)</f>
         <v/>
       </c>
-      <c r="V20" s="14" t="inlineStr"/>
+      <c r="V20" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: CI green, 8 tests (order, signals, sidecar death, fail-fast before sidecar). Combined wave-4 check pending.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3515,19 +3627,27 @@
         <f>IF(OR(I21="",L21=""),"",I21*L21)</f>
         <v/>
       </c>
-      <c r="N21" s="13" t="n"/>
-      <c r="O21" s="13" t="n"/>
+      <c r="N21" s="26" t="n">
+        <v>46314.57450231481</v>
+      </c>
+      <c r="O21" s="26" t="n">
+        <v>46314.57635416667</v>
+      </c>
       <c r="P21" s="7">
         <f>IF(AND(ISNUMBER(N21),ISNUMBER(O21)),ROUND((O21-N21)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" s="14" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="R21" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/24</t>
+        </is>
+      </c>
       <c r="S21" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T21" s="5">
@@ -3538,7 +3658,11 @@
         <f>IF(OR(T21="",L21=""),"",T21/L21)</f>
         <v/>
       </c>
-      <c r="V21" s="14" t="inlineStr"/>
+      <c r="V21" s="6" t="inlineStr">
+        <is>
+          <t>Accepted attempt 2: guarded drive_list under new 'list' step (schema.ts STEPS), 7 tests, CI green, merged #24. Real-runtime check conforms once guard logs caller's step (Quinn follow-up) and #26 lands.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3701,18 +3825,18 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>T1.2</t>
+          <t>T5.1</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S5</t>
         </is>
       </c>
       <c r="C24" s="15" t="n"/>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Rowan</t>
+          <t>Ellis</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
@@ -3741,10 +3865,10 @@
         <v/>
       </c>
       <c r="N24" s="26" t="n">
-        <v>46314.54398148148</v>
+        <v>46314.54443287037</v>
       </c>
       <c r="O24" s="26" t="n">
-        <v>46314.54516203704</v>
+        <v>46314.54645833333</v>
       </c>
       <c r="P24" s="7">
         <f>IF(AND(ISNUMBER(N24),ISNUMBER(O24)),ROUND((O24-N24)*1440,1),"")</f>
@@ -3752,7 +3876,11 @@
       </c>
       <c r="Q24" s="14" t="n"/>
       <c r="R24" s="14" t="n"/>
-      <c r="S24" s="14" t="n"/>
+      <c r="S24" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="T24" s="5">
         <f>IF(S24="Y",SUMIFS($P$2:$P$62,$A$2:$A$62,A24&amp;"")/20,"")</f>
         <v/>
@@ -3763,22 +3891,44 @@
       </c>
       <c r="V24" s="6" t="inlineStr">
         <is>
-          <t>Earlier work segment of the accepted attempt (paused while blocked).</t>
+          <t>Original attempt: later found defective (sample fixture keyed to seed-10 hash; tests wrote into committed fixture) - superseded by rework.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="n"/>
-      <c r="B25" s="15" t="n"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>T1.2</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
       <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="15" t="n"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Rowan</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="F25" s="15" t="n"/>
       <c r="G25" s="15" t="n"/>
       <c r="H25" s="15" t="n"/>
       <c r="I25" s="5" t="n"/>
-      <c r="J25" s="15" t="n"/>
-      <c r="K25" s="15" t="n"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
       <c r="L25" s="4">
         <f>IF(J25="","",INDEX(Calibration!$D$5:$D$11,MATCH(J25&amp;" "&amp;K25,Calibration!$A$5:$A$11,0)))</f>
         <v/>
@@ -3787,8 +3937,12 @@
         <f>IF(OR(I25="",L25=""),"",I25*L25)</f>
         <v/>
       </c>
-      <c r="N25" s="13" t="n"/>
-      <c r="O25" s="13" t="n"/>
+      <c r="N25" s="26" t="n">
+        <v>46314.54398148148</v>
+      </c>
+      <c r="O25" s="26" t="n">
+        <v>46314.54516203704</v>
+      </c>
       <c r="P25" s="7">
         <f>IF(AND(ISNUMBER(N25),ISNUMBER(O25)),ROUND((O25-N25)*1440,1),"")</f>
         <v/>
@@ -3804,20 +3958,46 @@
         <f>IF(OR(T25="",L25=""),"",T25/L25)</f>
         <v/>
       </c>
-      <c r="V25" s="14" t="n"/>
+      <c r="V25" s="6" t="inlineStr">
+        <is>
+          <t>Earlier work segment of the accepted attempt (paused while blocked).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="n"/>
-      <c r="B26" s="15" t="n"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>T8.2</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
       <c r="C26" s="15" t="n"/>
-      <c r="D26" s="15" t="n"/>
-      <c r="E26" s="15" t="n"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Mika</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="F26" s="15" t="n"/>
       <c r="G26" s="15" t="n"/>
       <c r="H26" s="15" t="n"/>
       <c r="I26" s="5" t="n"/>
-      <c r="J26" s="15" t="n"/>
-      <c r="K26" s="15" t="n"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Sonnet 5.5</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
       <c r="L26" s="4">
         <f>IF(J26="","",INDEX(Calibration!$D$5:$D$11,MATCH(J26&amp;" "&amp;K26,Calibration!$A$5:$A$11,0)))</f>
         <v/>
@@ -3826,14 +4006,22 @@
         <f>IF(OR(I26="",L26=""),"",I26*L26)</f>
         <v/>
       </c>
-      <c r="N26" s="13" t="n"/>
-      <c r="O26" s="13" t="n"/>
+      <c r="N26" s="26" t="n">
+        <v>46314.57449074074</v>
+      </c>
+      <c r="O26" s="26" t="n">
+        <v>46314.57518518518</v>
+      </c>
       <c r="P26" s="7">
         <f>IF(AND(ISNUMBER(N26),ISNUMBER(O26)),ROUND((O26-N26)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q26" s="14" t="n"/>
-      <c r="R26" s="14" t="n"/>
+      <c r="R26" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/26</t>
+        </is>
+      </c>
       <c r="S26" s="14" t="n"/>
       <c r="T26" s="5">
         <f>IF(S26="Y",SUMIFS($P$2:$P$62,$A$2:$A$62,A26&amp;"")/20,"")</f>
@@ -3843,20 +4031,46 @@
         <f>IF(OR(T26="",L26=""),"",T26/L26)</f>
         <v/>
       </c>
-      <c r="V26" s="14" t="n"/>
+      <c r="V26" s="6" t="inlineStr">
+        <is>
+          <t>Follow-up (orchestrator request, not rework): expected list line for guarded drive_list (PR #26, merges after #24)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="n"/>
-      <c r="B27" s="15" t="n"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>T4.1</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
       <c r="C27" s="15" t="n"/>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="15" t="n"/>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Rowan</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="F27" s="15" t="n"/>
       <c r="G27" s="15" t="n"/>
       <c r="H27" s="15" t="n"/>
       <c r="I27" s="5" t="n"/>
-      <c r="J27" s="15" t="n"/>
-      <c r="K27" s="15" t="n"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
       <c r="L27" s="4">
         <f>IF(J27="","",INDEX(Calibration!$D$5:$D$11,MATCH(J27&amp;" "&amp;K27,Calibration!$A$5:$A$11,0)))</f>
         <v/>
@@ -3865,14 +4079,22 @@
         <f>IF(OR(I27="",L27=""),"",I27*L27)</f>
         <v/>
       </c>
-      <c r="N27" s="13" t="n"/>
-      <c r="O27" s="13" t="n"/>
+      <c r="N27" s="26" t="n">
+        <v>46314.56958333333</v>
+      </c>
+      <c r="O27" s="26" t="n">
+        <v>46314.57152777778</v>
+      </c>
       <c r="P27" s="7">
         <f>IF(AND(ISNUMBER(N27),ISNUMBER(O27)),ROUND((O27-N27)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q27" s="14" t="n"/>
-      <c r="R27" s="14" t="n"/>
+      <c r="R27" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/21</t>
+        </is>
+      </c>
       <c r="S27" s="14" t="n"/>
       <c r="T27" s="5">
         <f>IF(S27="Y",SUMIFS($P$2:$P$62,$A$2:$A$62,A27&amp;"")/20,"")</f>
@@ -3882,20 +4104,46 @@
         <f>IF(OR(T27="",L27=""),"",T27/L27)</f>
         <v/>
       </c>
-      <c r="V27" s="14" t="n"/>
+      <c r="V27" s="6" t="inlineStr">
+        <is>
+          <t>Follow-up (orchestrator request, not rework): wire Drive factory into reset/drop (PR #21)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="n"/>
-      <c r="B28" s="15" t="n"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>T10.2</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
       <c r="C28" s="15" t="n"/>
-      <c r="D28" s="15" t="n"/>
-      <c r="E28" s="15" t="n"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Quinn</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="F28" s="15" t="n"/>
       <c r="G28" s="15" t="n"/>
       <c r="H28" s="15" t="n"/>
       <c r="I28" s="5" t="n"/>
-      <c r="J28" s="15" t="n"/>
-      <c r="K28" s="15" t="n"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
       <c r="L28" s="4">
         <f>IF(J28="","",INDEX(Calibration!$D$5:$D$11,MATCH(J28&amp;" "&amp;K28,Calibration!$A$5:$A$11,0)))</f>
         <v/>
@@ -3904,14 +4152,22 @@
         <f>IF(OR(I28="",L28=""),"",I28*L28)</f>
         <v/>
       </c>
-      <c r="N28" s="13" t="n"/>
-      <c r="O28" s="13" t="n"/>
+      <c r="N28" s="26" t="n">
+        <v>46314.57690972222</v>
+      </c>
+      <c r="O28" s="26" t="n">
+        <v>46314.57835648148</v>
+      </c>
       <c r="P28" s="7">
         <f>IF(AND(ISNUMBER(N28),ISNUMBER(O28)),ROUND((O28-N28)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q28" s="14" t="n"/>
-      <c r="R28" s="14" t="n"/>
+      <c r="R28" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/27</t>
+        </is>
+      </c>
       <c r="S28" s="14" t="n"/>
       <c r="T28" s="5">
         <f>IF(S28="Y",SUMIFS($P$2:$P$62,$A$2:$A$62,A28&amp;"")/20,"")</f>
@@ -3921,20 +4177,46 @@
         <f>IF(OR(T28="",L28=""),"",T28/L28)</f>
         <v/>
       </c>
-      <c r="V28" s="14" t="n"/>
+      <c r="V28" s="6" t="inlineStr">
+        <is>
+          <t>Follow-up (orchestrator request, not rework): guard logs caller's step for drive_list (PR #27)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="n"/>
-      <c r="B29" s="15" t="n"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>T6.1</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
       <c r="C29" s="15" t="n"/>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="15" t="n"/>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Noor</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="F29" s="15" t="n"/>
       <c r="G29" s="15" t="n"/>
       <c r="H29" s="15" t="n"/>
       <c r="I29" s="5" t="n"/>
-      <c r="J29" s="15" t="n"/>
-      <c r="K29" s="15" t="n"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
       <c r="L29" s="4">
         <f>IF(J29="","",INDEX(Calibration!$D$5:$D$11,MATCH(J29&amp;" "&amp;K29,Calibration!$A$5:$A$11,0)))</f>
         <v/>
@@ -3943,8 +4225,12 @@
         <f>IF(OR(I29="",L29=""),"",I29*L29)</f>
         <v/>
       </c>
-      <c r="N29" s="13" t="n"/>
-      <c r="O29" s="13" t="n"/>
+      <c r="N29" s="26" t="n">
+        <v>46314.56981481481</v>
+      </c>
+      <c r="O29" s="26" t="n">
+        <v>46314.57160879629</v>
+      </c>
       <c r="P29" s="7">
         <f>IF(AND(ISNUMBER(N29),ISNUMBER(O29)),ROUND((O29-N29)*1440,1),"")</f>
         <v/>
@@ -3960,20 +4246,46 @@
         <f>IF(OR(T29="",L29=""),"",T29/L29)</f>
         <v/>
       </c>
-      <c r="V29" s="14" t="n"/>
+      <c r="V29" s="6" t="inlineStr">
+        <is>
+          <t>Earlier work segment of the accepted attempt (paused while blocked).</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="n"/>
-      <c r="B30" s="15" t="n"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>T12.1</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
       <c r="C30" s="15" t="n"/>
-      <c r="D30" s="15" t="n"/>
-      <c r="E30" s="15" t="n"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Rowan</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="F30" s="15" t="n"/>
       <c r="G30" s="15" t="n"/>
       <c r="H30" s="15" t="n"/>
       <c r="I30" s="5" t="n"/>
-      <c r="J30" s="15" t="n"/>
-      <c r="K30" s="15" t="n"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
       <c r="L30" s="4">
         <f>IF(J30="","",INDEX(Calibration!$D$5:$D$11,MATCH(J30&amp;" "&amp;K30,Calibration!$A$5:$A$11,0)))</f>
         <v/>
@@ -3982,15 +4294,23 @@
         <f>IF(OR(I30="",L30=""),"",I30*L30)</f>
         <v/>
       </c>
-      <c r="N30" s="13" t="n"/>
-      <c r="O30" s="13" t="n"/>
+      <c r="N30" s="26" t="n">
+        <v>46314.57152777778</v>
+      </c>
+      <c r="O30" s="26" t="n">
+        <v>46314.5738425926</v>
+      </c>
       <c r="P30" s="7">
         <f>IF(AND(ISNUMBER(N30),ISNUMBER(O30)),ROUND((O30-N30)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q30" s="14" t="n"/>
       <c r="R30" s="14" t="n"/>
-      <c r="S30" s="14" t="n"/>
+      <c r="S30" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="T30" s="5">
         <f>IF(S30="Y",SUMIFS($P$2:$P$62,$A$2:$A$62,A30&amp;"")/20,"")</f>
         <v/>
@@ -3999,7 +4319,11 @@
         <f>IF(OR(T30="",L30=""),"",T30/L30)</f>
         <v/>
       </c>
-      <c r="V30" s="14" t="n"/>
+      <c r="V30" s="6" t="inlineStr">
+        <is>
+          <t>Rejected attempt 1: agent discovered Legal files via unguarded DriveClient.list to fit expected file; orchestrator requires guarded drive_list under new 'list' step.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="n"/>
@@ -6357,7 +6681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6384,6 +6708,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -6873,6 +7198,7 @@
       </c>
       <c r="H18" s="8" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="19" t="inlineStr">
         <is>
@@ -7119,6 +7445,7 @@
         <v/>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
         <is>
@@ -7231,6 +7558,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="25" t="inlineStr">
         <is>
@@ -7343,21 +7671,45 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="25" t="inlineStr">
+        <is>
+          <t>Poller durability: if the log write fails after a successful move, that classify line is lost. Persist pending lines and retry them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="25" t="inlineStr">
+        <is>
+          <t>A wider confidence margin for seed 10. It records at 0.66 against the 0.70 threshold, so a live re-record could cross it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="25" t="inlineStr">
+        <is>
+          <t>A faster reset on Workspace Drive (batch calls); today it takes 23–45 s.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="18">
+    <mergeCell ref="A50:H50"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A46:H46"/>
     <mergeCell ref="A35:H35"/>
     <mergeCell ref="A43:H43"/>
     <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A42:H42"/>
     <mergeCell ref="A41:H41"/>
-    <mergeCell ref="A36:H36"/>
     <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A46:H46"/>
     <mergeCell ref="A37:H37"/>
     <mergeCell ref="A40:H40"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: phase 4 acceptance, demo run logs and final actuals
Two runs from a clean Drive: compare identical, both match expected.
All 12 stories done; workbook actuals and calibration final.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/Hashirai Clearance POC - Plan.xlsx
+++ b/planning/Hashirai Clearance POC - Plan.xlsx
@@ -1145,12 +1145,12 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L8" s="7">
@@ -1214,12 +1214,12 @@
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L9" s="7">
@@ -1490,12 +1490,12 @@
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="L13" s="7">
@@ -3724,19 +3724,27 @@
         <f>IF(OR(I22="",L22=""),"",I22*L22)</f>
         <v/>
       </c>
-      <c r="N22" s="13" t="n"/>
-      <c r="O22" s="13" t="n"/>
+      <c r="N22" s="26" t="n">
+        <v>46314.57934027778</v>
+      </c>
+      <c r="O22" s="26" t="n">
+        <v>46314.58083333333</v>
+      </c>
       <c r="P22" s="7">
         <f>IF(AND(ISNUMBER(N22),ISNUMBER(O22)),ROUND((O22-N22)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="R22" s="6" t="inlineStr">
+        <is>
+          <t>https://github.com/soham956/OpenAPPA/pull/29</t>
+        </is>
+      </c>
       <c r="S22" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="T22" s="5">
@@ -3747,7 +3755,11 @@
         <f>IF(OR(T22="",L22=""),"",T22/L22)</f>
         <v/>
       </c>
-      <c r="V22" s="14" t="inlineStr"/>
+      <c r="V22" s="6" t="inlineStr">
+        <is>
+          <t>Accepted: e2e step 2 against real appa + fake Drive, conforms to expected (11 enforce + 1 outbox), second run identical, ran in CI (not skipped).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(planning): log post-acceptance rework; review items to Later
T3.1 rework (Sasha, drive timeouts, #32) and T10.2 rework (Quinn,
review C2/C6, #33) logged per agent. Deferred review findings added
to the Later list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planning/Hashirai Clearance POC - Plan.xlsx
+++ b/planning/Hashirai Clearance POC - Plan.xlsx
@@ -2173,21 +2173,21 @@
         <v/>
       </c>
       <c r="N6" s="26" t="n">
-        <v>46314.54443287037</v>
+        <v>46314.61380787037</v>
       </c>
       <c r="O6" s="26" t="n">
-        <v>46314.54755787037</v>
+        <v>46314.61740740741</v>
       </c>
       <c r="P6" s="7">
         <f>IF(AND(ISNUMBER(N6),ISNUMBER(O6)),ROUND((O6-N6)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q6" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R6" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/soham956/OpenAPPA/pull/9</t>
+          <t>https://github.com/soham956/OpenAPPA/pull/9 + #32 (rework)</t>
         </is>
       </c>
       <c r="S6" s="6" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="V6" s="6" t="inlineStr">
         <is>
-          <t>Accepted: in scope (5 files), contract suite runs on fake and Google stub, trash is soft (trashed=true), DriveScopeError outside the tree. Combined wave-2 check passed (128/128).</t>
+          <t>Accepted after rework (PR #32): 20 s request timeouts, safe retries (idempotent reads; move/trash verify-then-retry; upload never retried). Found by orchestrator during the live recording rehearsal.</t>
         </is>
       </c>
     </row>
@@ -3143,21 +3143,21 @@
         <v/>
       </c>
       <c r="N16" s="26" t="n">
-        <v>46314.5622337963</v>
+        <v>46314.63260416667</v>
       </c>
       <c r="O16" s="26" t="n">
-        <v>46314.5671412037</v>
+        <v>46314.63730324074</v>
       </c>
       <c r="P16" s="7">
         <f>IF(AND(ISNUMBER(N16),ISNUMBER(O16)),ROUND((O16-N16)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R16" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/soham956/OpenAPPA/pull/20</t>
+          <t>https://github.com/soham956/OpenAPPA/pull/20 + #27 (follow-up) + #33 (rework)</t>
         </is>
       </c>
       <c r="S16" s="6" t="inlineStr">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="V16" s="6" t="inlineStr">
         <is>
-          <t>Accepted: exact 2a/2b/2c reasons live + replayed from fixtures; denied tools never run; CI ran live guard tests. Combined wave-3 check 220/220. Has its own default drive tools - T12.1 to inject T11.2's.</t>
+          <t>Accepted after rework (PR #33): fail closed on folder change (C2), Guard.call total (C6); 262 tests incl. live; demo unchanged.</t>
         </is>
       </c>
     </row>
@@ -3910,18 +3910,18 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>T1.2</t>
+          <t>T3.1</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="C25" s="15" t="n"/>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Rowan</t>
+          <t>Sasha</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
@@ -3950,10 +3950,10 @@
         <v/>
       </c>
       <c r="N25" s="26" t="n">
-        <v>46314.54398148148</v>
+        <v>46314.54443287037</v>
       </c>
       <c r="O25" s="26" t="n">
-        <v>46314.54516203704</v>
+        <v>46314.54755787037</v>
       </c>
       <c r="P25" s="7">
         <f>IF(AND(ISNUMBER(N25),ISNUMBER(O25)),ROUND((O25-N25)*1440,1),"")</f>
@@ -3961,7 +3961,11 @@
       </c>
       <c r="Q25" s="14" t="n"/>
       <c r="R25" s="14" t="n"/>
-      <c r="S25" s="14" t="n"/>
+      <c r="S25" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="T25" s="5">
         <f>IF(S25="Y",SUMIFS($P$2:$P$62,$A$2:$A$62,A25&amp;"")/20,"")</f>
         <v/>
@@ -3972,29 +3976,29 @@
       </c>
       <c r="V25" s="6" t="inlineStr">
         <is>
-          <t>Earlier work segment of the accepted attempt (paused while blocked).</t>
+          <t>Original attempt: later found defective (no Drive request timeouts - a hung call stalled the live demo poller) - superseded by rework.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>T8.2</t>
+          <t>T1.2</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>S8</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="C26" s="15" t="n"/>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Mika</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" s="15" t="n"/>
       <c r="G26" s="15" t="n"/>
@@ -4002,7 +4006,7 @@
       <c r="I26" s="5" t="n"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Sonnet 5.5</t>
+          <t>Opus 5.5</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -4019,21 +4023,17 @@
         <v/>
       </c>
       <c r="N26" s="26" t="n">
-        <v>46314.57449074074</v>
+        <v>46314.54398148148</v>
       </c>
       <c r="O26" s="26" t="n">
-        <v>46314.57518518518</v>
+        <v>46314.54516203704</v>
       </c>
       <c r="P26" s="7">
         <f>IF(AND(ISNUMBER(N26),ISNUMBER(O26)),ROUND((O26-N26)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q26" s="14" t="n"/>
-      <c r="R26" s="6" t="inlineStr">
-        <is>
-          <t>https://github.com/soham956/OpenAPPA/pull/26</t>
-        </is>
-      </c>
+      <c r="R26" s="6" t="n"/>
       <c r="S26" s="14" t="n"/>
       <c r="T26" s="5">
         <f>IF(S26="Y",SUMIFS($P$2:$P$62,$A$2:$A$62,A26&amp;"")/20,"")</f>
@@ -4045,25 +4045,25 @@
       </c>
       <c r="V26" s="6" t="inlineStr">
         <is>
-          <t>Follow-up (orchestrator request, not rework): expected list line for guarded drive_list (PR #26, merges after #24)</t>
+          <t>Earlier work segment of the accepted attempt (paused while blocked).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>T4.1</t>
+          <t>T8.2</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S8</t>
         </is>
       </c>
       <c r="C27" s="15" t="n"/>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Rowan</t>
+          <t>Mika</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
@@ -4075,7 +4075,7 @@
       <c r="I27" s="5" t="n"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Opus 5.5</t>
+          <t>Sonnet 5.5</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -4092,10 +4092,10 @@
         <v/>
       </c>
       <c r="N27" s="26" t="n">
-        <v>46314.56958333333</v>
+        <v>46314.57449074074</v>
       </c>
       <c r="O27" s="26" t="n">
-        <v>46314.57152777778</v>
+        <v>46314.57518518518</v>
       </c>
       <c r="P27" s="7">
         <f>IF(AND(ISNUMBER(N27),ISNUMBER(O27)),ROUND((O27-N27)*1440,1),"")</f>
@@ -4104,7 +4104,7 @@
       <c r="Q27" s="14" t="n"/>
       <c r="R27" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/soham956/OpenAPPA/pull/21</t>
+          <t>https://github.com/soham956/OpenAPPA/pull/26</t>
         </is>
       </c>
       <c r="S27" s="14" t="n"/>
@@ -4118,25 +4118,25 @@
       </c>
       <c r="V27" s="6" t="inlineStr">
         <is>
-          <t>Follow-up (orchestrator request, not rework): wire Drive factory into reset/drop (PR #21)</t>
+          <t>Follow-up (orchestrator request, not rework): expected list line for guarded drive_list (PR #26, merges after #24)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>T10.2</t>
+          <t>T4.1</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="C28" s="15" t="n"/>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Quinn</t>
+          <t>Rowan</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="L28" s="4">
@@ -4165,10 +4165,10 @@
         <v/>
       </c>
       <c r="N28" s="26" t="n">
-        <v>46314.57690972222</v>
+        <v>46314.56958333333</v>
       </c>
       <c r="O28" s="26" t="n">
-        <v>46314.57835648148</v>
+        <v>46314.57152777778</v>
       </c>
       <c r="P28" s="7">
         <f>IF(AND(ISNUMBER(N28),ISNUMBER(O28)),ROUND((O28-N28)*1440,1),"")</f>
@@ -4177,7 +4177,7 @@
       <c r="Q28" s="14" t="n"/>
       <c r="R28" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/soham956/OpenAPPA/pull/27</t>
+          <t>https://github.com/soham956/OpenAPPA/pull/21</t>
         </is>
       </c>
       <c r="S28" s="14" t="n"/>
@@ -4191,29 +4191,29 @@
       </c>
       <c r="V28" s="6" t="inlineStr">
         <is>
-          <t>Follow-up (orchestrator request, not rework): guard logs caller's step for drive_list (PR #27)</t>
+          <t>Follow-up (orchestrator request, not rework): wire Drive factory into reset/drop (PR #21)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>T6.1</t>
+          <t>T10.2</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>S6</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="C29" s="15" t="n"/>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Noor</t>
+          <t>Quinn</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F29" s="15" t="n"/>
       <c r="G29" s="15" t="n"/>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="L29" s="4">
@@ -4238,10 +4238,10 @@
         <v/>
       </c>
       <c r="N29" s="26" t="n">
-        <v>46314.56981481481</v>
+        <v>46314.5622337963</v>
       </c>
       <c r="O29" s="26" t="n">
-        <v>46314.57160879629</v>
+        <v>46314.5671412037</v>
       </c>
       <c r="P29" s="7">
         <f>IF(AND(ISNUMBER(N29),ISNUMBER(O29)),ROUND((O29-N29)*1440,1),"")</f>
@@ -4249,7 +4249,11 @@
       </c>
       <c r="Q29" s="14" t="n"/>
       <c r="R29" s="14" t="n"/>
-      <c r="S29" s="14" t="n"/>
+      <c r="S29" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="T29" s="5">
         <f>IF(S29="Y",SUMIFS($P$2:$P$62,$A$2:$A$62,A29&amp;"")/20,"")</f>
         <v/>
@@ -4260,25 +4264,25 @@
       </c>
       <c r="V29" s="6" t="inlineStr">
         <is>
-          <t>Earlier work segment of the accepted attempt (paused while blocked).</t>
+          <t>Original attempt: later found defective by independent code review (C2 check-then-read race; C6 Guard.call could throw and skip logging) - superseded by rework.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>T12.1</t>
+          <t>T6.1</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S6</t>
         </is>
       </c>
       <c r="C30" s="15" t="n"/>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Rowan</t>
+          <t>Noor</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
@@ -4295,7 +4299,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="L30" s="4">
@@ -4307,10 +4311,10 @@
         <v/>
       </c>
       <c r="N30" s="26" t="n">
-        <v>46314.57152777778</v>
+        <v>46314.56981481481</v>
       </c>
       <c r="O30" s="26" t="n">
-        <v>46314.5738425926</v>
+        <v>46314.57160879629</v>
       </c>
       <c r="P30" s="7">
         <f>IF(AND(ISNUMBER(N30),ISNUMBER(O30)),ROUND((O30-N30)*1440,1),"")</f>
@@ -4318,11 +4322,7 @@
       </c>
       <c r="Q30" s="14" t="n"/>
       <c r="R30" s="14" t="n"/>
-      <c r="S30" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="S30" s="6" t="n"/>
       <c r="T30" s="5">
         <f>IF(S30="Y",SUMIFS($P$2:$P$62,$A$2:$A$62,A30&amp;"")/20,"")</f>
         <v/>
@@ -4333,22 +4333,44 @@
       </c>
       <c r="V30" s="6" t="inlineStr">
         <is>
-          <t>Rejected attempt 1: agent discovered Legal files via unguarded DriveClient.list to fit expected file; orchestrator requires guarded drive_list under new 'list' step.</t>
+          <t>Earlier work segment of the accepted attempt (paused while blocked).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="15" t="n"/>
-      <c r="B31" s="15" t="n"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>T12.1</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
       <c r="C31" s="15" t="n"/>
-      <c r="D31" s="15" t="n"/>
-      <c r="E31" s="15" t="n"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Rowan</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="F31" s="15" t="n"/>
       <c r="G31" s="15" t="n"/>
       <c r="H31" s="15" t="n"/>
       <c r="I31" s="5" t="n"/>
-      <c r="J31" s="15" t="n"/>
-      <c r="K31" s="15" t="n"/>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Opus 5.5</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
       <c r="L31" s="4">
         <f>IF(J31="","",INDEX(Calibration!$D$5:$D$11,MATCH(J31&amp;" "&amp;K31,Calibration!$A$5:$A$11,0)))</f>
         <v/>
@@ -4357,15 +4379,23 @@
         <f>IF(OR(I31="",L31=""),"",I31*L31)</f>
         <v/>
       </c>
-      <c r="N31" s="13" t="n"/>
-      <c r="O31" s="13" t="n"/>
+      <c r="N31" s="26" t="n">
+        <v>46314.57152777778</v>
+      </c>
+      <c r="O31" s="26" t="n">
+        <v>46314.5738425926</v>
+      </c>
       <c r="P31" s="7">
         <f>IF(AND(ISNUMBER(N31),ISNUMBER(O31)),ROUND((O31-N31)*1440,1),"")</f>
         <v/>
       </c>
       <c r="Q31" s="14" t="n"/>
       <c r="R31" s="14" t="n"/>
-      <c r="S31" s="14" t="n"/>
+      <c r="S31" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="T31" s="5">
         <f>IF(S31="Y",SUMIFS($P$2:$P$62,$A$2:$A$62,A31&amp;"")/20,"")</f>
         <v/>
@@ -4374,7 +4404,11 @@
         <f>IF(OR(T31="",L31=""),"",T31/L31)</f>
         <v/>
       </c>
-      <c r="V31" s="14" t="n"/>
+      <c r="V31" s="6" t="inlineStr">
+        <is>
+          <t>Rejected attempt 1: agent discovered Legal files via unguarded DriveClient.list to fit expected file; orchestrator requires guarded drive_list under new 'list' step.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="15" t="n"/>
@@ -6693,7 +6727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7630,7 +7664,7 @@
     <row r="41">
       <c r="A41" s="25" t="inlineStr">
         <is>
-          <t>Per-team audiences (an Accounting list separate from `internal`).</t>
+          <t>Per-team audiences (an Accounting list separate from internal).</t>
         </is>
       </c>
     </row>
@@ -7704,26 +7738,138 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="25" t="inlineStr">
+        <is>
+          <t>From the code review (docs/poc-review.md), must-fix before building on this:</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – C1: run the guard outside the agent's process, bound to one trajectory per connection, with unique root ids.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – C3: one source of truth for labels: store the label per file ID and revision, or lock folder writes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – C4: put classifier egress to TypeSafe under policy, and stop writing fixtures at run time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – C5: attachments become file IDs that the guard reads and labels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
+          <t>From the code review, should-fix:</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – C7: an outcome for "ran, settle failed".</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – C8: typed offers and reasons instead of matching runtime text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – C9: a service account scoped to the tree, and a guarded token listener.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – Q1: remove the duplicated Drive tools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – Q2: generate the policy knowledge from appa describe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – Q3: take the demo enums out of the core types.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – Q5: shared atomic writes and a memory lock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      – Q6: fewer Drive calls per read.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A50:H50"/>
+  <mergeCells count="32">
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A39:H39"/>
-    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A59:H59"/>
     <mergeCell ref="A51:H51"/>
-    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A64:H64"/>
+    <mergeCell ref="A60:H60"/>
     <mergeCell ref="A36:H36"/>
     <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A61:H61"/>
+    <mergeCell ref="A65:H65"/>
+    <mergeCell ref="A54:H54"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A56:H56"/>
+    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A42:H42"/>
     <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A53:H53"/>
     <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A63:H63"/>
     <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A58:H58"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>